<commit_message>
version test 1 only fix data from box
</commit_message>
<xml_diff>
--- a/Aji_game copy_April.xlsx
+++ b/Aji_game copy_April.xlsx
@@ -1350,336 +1350,8 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-TH"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'gameplay_report(score) '!$B$1</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="C00000"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:dLbls>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="C00000"/>
-              </a:solidFill>
-              <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-                <a:solidFill>
-                  <a:schemeClr val="accent3"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-                <a:miter lim="800000"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="bg1"/>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-TH"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="t"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:numRef>
-              <c:f>'gameplay_report(score) '!$A$126:$A$147</c:f>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'gameplay_report(score) '!$B$126:$B$147</c:f>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6386-F942-8A1B-A2D1B6C2E5A6}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="t"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:marker val="1"/>
-        <c:smooth val="0"/>
-        <c:axId val="1311679680"/>
-        <c:axId val="1351481792"/>
-      </c:lineChart>
-      <c:dateAx>
-        <c:axId val="1311679680"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="m/d/yy" sourceLinked="1"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-TH"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1351481792"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblOffset val="100"/>
-        <c:baseTimeUnit val="days"/>
-      </c:dateAx>
-      <c:valAx>
-        <c:axId val="1351481792"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="0,&quot;k&quot;" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-TH"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1311679680"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-TH"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart"><c:date1904 val="0"/><c:lang val="en-US"/><c:roundedCorners val="0"/><mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006"><mc:Choice Requires="c14" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart"><c14:style val="102"/></mc:Choice><mc:Fallback><c:style val="2"/></mc:Fallback></mc:AlternateContent><c:chart><c:title><c:overlay val="0"/><c:spPr><a:noFill/><a:ln><a:noFill/></a:ln><a:effectLst/></c:spPr><c:txPr><a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/><a:lstStyle/><a:p><a:pPr><a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="65000"/><a:lumOff val="35000"/></a:schemeClr></a:solidFill><a:latin typeface="+mn-lt"/><a:ea typeface="+mn-ea"/><a:cs typeface="+mn-cs"/></a:defRPr></a:pPr><a:endParaRPr lang="en-TH"/></a:p></c:txPr></c:title><c:autoTitleDeleted val="0"/><c:plotArea><c:layout/><c:lineChart><c:grouping val="standard"/><c:varyColors val="0"/><c:ser><c:idx val="0"/><c:order val="0"/><c:tx><c:strRef><c:f>'gameplay_report(score) '!$B$1</c:f></c:strRef></c:tx><c:spPr><a:ln w="28575" cap="rnd"><a:solidFill><a:schemeClr val="accent3"/></a:solidFill><a:round/></a:ln><a:effectLst/></c:spPr><c:marker><c:symbol val="circle"/><c:size val="5"/><c:spPr><a:solidFill><a:schemeClr val="accent3"/></a:solidFill><a:ln w="9525"><a:solidFill><a:schemeClr val="accent3"/></a:solidFill></a:ln><a:effectLst/></c:spPr></c:marker><c:dLbls><c:spPr><a:solidFill><a:schemeClr val="accent3"/></a:solidFill><a:ln w="19050" cap="flat" cmpd="sng" algn="ctr"><a:solidFill><a:schemeClr val="accent3"/></a:solidFill><a:prstDash val="solid"/><a:miter lim="800000"/></a:ln><a:effectLst/></c:spPr><c:txPr><a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"><a:spAutoFit/></a:bodyPr><a:lstStyle/><a:p><a:pPr><a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"><a:solidFill><a:schemeClr val="bg1"/></a:solidFill><a:latin typeface="+mn-lt"/><a:ea typeface="+mn-ea"/><a:cs typeface="+mn-cs"/></a:defRPr></a:pPr><a:endParaRPr lang="en-TH"/></a:p></c:txPr><c:dLblPos val="t"/><c:showLegendKey val="0"/><c:showVal val="1"/><c:showCatName val="0"/><c:showSerName val="0"/><c:showPercent val="0"/><c:showBubbleSize val="0"/><c:showLeaderLines val="0"/><c:extLst><c:ext uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}" xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart"><c15:showLeaderLines val="1"/><c15:leaderLines><c:spPr><a:ln w="9525" cap="flat" cmpd="sng" algn="ctr"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="35000"/><a:lumOff val="65000"/></a:schemeClr></a:solidFill><a:round/></a:ln><a:effectLst/></c:spPr></c15:leaderLines></c:ext></c:extLst></c:dLbls><c:cat><c:numRef><c:f>'gameplay_report(score) '!$A$67:$A$94</c:f></c:numRef></c:cat><c:val><c:numRef><c:f>'gameplay_report(score) '!$B$67:$B$94</c:f></c:numRef></c:val><c:smooth val="0"/><c:extLst><c:ext uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}" xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart"><c16:uniqueId val="{00000000-6386-F942-8A1B-A2D1B6C2E5A6}"/></c:ext></c:extLst></c:ser><c:dLbls><c:dLblPos val="t"/><c:showLegendKey val="0"/><c:showVal val="1"/><c:showCatName val="0"/><c:showSerName val="0"/><c:showPercent val="0"/><c:showBubbleSize val="0"/></c:dLbls><c:marker val="1"/><c:smooth val="0"/><c:axId val="1311679680"/><c:axId val="1351481792"/></c:lineChart><c:dateAx><c:axId val="1311679680"/><c:scaling><c:orientation val="minMax"/></c:scaling><c:delete val="0"/><c:axPos val="b"/><c:numFmt formatCode="m/d/yy" sourceLinked="1"/><c:majorTickMark val="out"/><c:minorTickMark val="none"/><c:tickLblPos val="nextTo"/><c:spPr><a:noFill/><a:ln w="9525" cap="flat" cmpd="sng" algn="ctr"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="15000"/><a:lumOff val="85000"/></a:schemeClr></a:solidFill><a:round/></a:ln><a:effectLst/></c:spPr><c:txPr><a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/><a:lstStyle/><a:p><a:pPr><a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="65000"/><a:lumOff val="35000"/></a:schemeClr></a:solidFill><a:latin typeface="+mn-lt"/><a:ea typeface="+mn-ea"/><a:cs typeface="+mn-cs"/></a:defRPr></a:pPr><a:endParaRPr lang="en-TH"/></a:p></c:txPr><c:crossAx val="1351481792"/><c:crosses val="autoZero"/><c:auto val="1"/><c:lblOffset val="100"/><c:baseTimeUnit val="days"/></c:dateAx><c:valAx><c:axId val="1351481792"/><c:scaling><c:orientation val="minMax"/></c:scaling><c:delete val="0"/><c:axPos val="l"/><c:majorGridlines><c:spPr><a:ln w="9525" cap="flat" cmpd="sng" algn="ctr"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="15000"/><a:lumOff val="85000"/></a:schemeClr></a:solidFill><a:round/></a:ln><a:effectLst/></c:spPr></c:majorGridlines><c:numFmt formatCode="0,&quot;k&quot;" sourceLinked="1"/><c:majorTickMark val="none"/><c:minorTickMark val="none"/><c:tickLblPos val="nextTo"/><c:spPr><a:noFill/><a:ln><a:noFill/></a:ln><a:effectLst/></c:spPr><c:txPr><a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/><a:lstStyle/><a:p><a:pPr><a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="65000"/><a:lumOff val="35000"/></a:schemeClr></a:solidFill><a:latin typeface="+mn-lt"/><a:ea typeface="+mn-ea"/><a:cs typeface="+mn-cs"/></a:defRPr></a:pPr><a:endParaRPr lang="en-TH"/></a:p></c:txPr><c:crossAx val="1311679680"/><c:crosses val="autoZero"/><c:crossBetween val="between"/></c:valAx><c:spPr><a:noFill/><a:ln><a:noFill/></a:ln><a:effectLst/></c:spPr></c:plotArea><c:plotVisOnly val="1"/><c:dispBlanksAs val="gap"/><c:showDLblsOverMax val="0"/><c:extLst><c:ext uri="{56B9EC1D-385E-4148-901F-78D8002777C0}" xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart"><c16r3:dataDisplayOptions16><c16r3:dispNaAsBlank val="1"/></c16r3:dataDisplayOptions16></c:ext></c:extLst></c:chart><c:spPr><a:solidFill><a:schemeClr val="bg1"/></a:solidFill><a:ln w="9525" cap="flat" cmpd="sng" algn="ctr"><a:solidFill><a:schemeClr val="tx1"><a:lumMod val="15000"/><a:lumOff val="85000"/></a:schemeClr></a:solidFill><a:round/></a:ln><a:effectLst/></c:spPr><c:txPr><a:bodyPr/><a:lstStyle/><a:p><a:pPr><a:defRPr/></a:pPr><a:endParaRPr lang="en-TH"/></a:p></c:txPr><c:printSettings><c:headerFooter/><c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/><c:pageSetup/></c:printSettings></c:chartSpace>ace>
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>